<commit_message>
add mayo, fix locations tags
</commit_message>
<xml_diff>
--- a/Database.xlsx
+++ b/Database.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6112e55300fcb9f7/Documents/FL_Studio/Music/Pink_Noise/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="84" documentId="8_{261B944D-3154-41C4-A810-0FE7F57DCA2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CD1BD070-D791-4ADD-9749-41A294B75CBF}"/>
+  <xr:revisionPtr revIDLastSave="87" documentId="8_{261B944D-3154-41C4-A810-0FE7F57DCA2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8A53BA6D-812C-446E-BEE2-C2D5EC75AA1A}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DFD942CF-3A3C-44FC-9CE1-5077A113D16C}"/>
   </bookViews>
@@ -434,9 +434,6 @@
     <t>https://jasonkahn.net/</t>
   </si>
   <si>
-    <t>Dublin, Leitrim</t>
-  </si>
-  <si>
     <t>Avant-garde, Noise</t>
   </si>
   <si>
@@ -449,9 +446,6 @@
     <t>Drone, Noise, Ambient</t>
   </si>
   <si>
-    <t>Sligo, Barcelona</t>
-  </si>
-  <si>
     <t>Avant-rock, Drone</t>
   </si>
   <si>
@@ -537,6 +531,12 @@
   </si>
   <si>
     <t>https://sexytadhg.bandcamp.com/album/sluttrad</t>
+  </si>
+  <si>
+    <t>Sligo/Barcelona</t>
+  </si>
+  <si>
+    <t>Dublin/Leitrim</t>
   </si>
 </sst>
 </file>
@@ -1246,7 +1246,7 @@
         <v>14</v>
       </c>
       <c r="C20" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>40</v>
@@ -1263,7 +1263,7 @@
         <v>43</v>
       </c>
       <c r="C21" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D21" t="s">
         <v>131</v>
@@ -1280,7 +1280,7 @@
         <v>6</v>
       </c>
       <c r="C22" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="D22" s="4" t="s">
         <v>45</v>
@@ -1305,13 +1305,13 @@
         <v>48</v>
       </c>
       <c r="B24" t="s">
+        <v>166</v>
+      </c>
+      <c r="C24" t="s">
         <v>132</v>
       </c>
-      <c r="C24" t="s">
+      <c r="D24" t="s">
         <v>133</v>
-      </c>
-      <c r="D24" t="s">
-        <v>134</v>
       </c>
       <c r="E24" t="s">
         <v>33</v>
@@ -1328,7 +1328,7 @@
         <v>50</v>
       </c>
       <c r="D25" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
@@ -1339,7 +1339,7 @@
         <v>52</v>
       </c>
       <c r="C26" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D26" s="4" t="s">
         <v>53</v>
@@ -1350,13 +1350,13 @@
         <v>54</v>
       </c>
       <c r="B27" t="s">
+        <v>165</v>
+      </c>
+      <c r="C27" t="s">
+        <v>136</v>
+      </c>
+      <c r="D27" t="s">
         <v>137</v>
-      </c>
-      <c r="C27" t="s">
-        <v>138</v>
-      </c>
-      <c r="D27" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
@@ -1367,7 +1367,7 @@
         <v>14</v>
       </c>
       <c r="C28" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D28" s="4" t="s">
         <v>57</v>
@@ -1381,10 +1381,10 @@
         <v>52</v>
       </c>
       <c r="C29" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D29" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
@@ -1395,10 +1395,10 @@
         <v>60</v>
       </c>
       <c r="C30" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="D30" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
@@ -1409,7 +1409,7 @@
         <v>55</v>
       </c>
       <c r="D31" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
@@ -1420,7 +1420,7 @@
         <v>52</v>
       </c>
       <c r="C32" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D32" s="4" t="s">
         <v>63</v>
@@ -1434,10 +1434,10 @@
         <v>6</v>
       </c>
       <c r="C33" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D33" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
@@ -1445,10 +1445,10 @@
         <v>65</v>
       </c>
       <c r="B34" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="C34" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="D34" s="4" t="s">
         <v>66</v>
@@ -1462,7 +1462,7 @@
         <v>20</v>
       </c>
       <c r="C35" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="D35" s="4" t="s">
         <v>68</v>
@@ -1473,10 +1473,10 @@
         <v>69</v>
       </c>
       <c r="B36" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C36" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="D36" s="4" t="s">
         <v>70</v>
@@ -1490,10 +1490,10 @@
         <v>52</v>
       </c>
       <c r="C37" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="D37" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
@@ -1504,10 +1504,10 @@
         <v>52</v>
       </c>
       <c r="C38" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="D38" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
@@ -1518,7 +1518,7 @@
         <v>52</v>
       </c>
       <c r="C39" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="D39" s="4" t="s">
         <v>74</v>
@@ -1532,7 +1532,7 @@
         <v>117</v>
       </c>
       <c r="D40" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
@@ -1543,7 +1543,7 @@
         <v>52</v>
       </c>
       <c r="C41" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="D41" s="4" t="s">
         <v>77</v>
@@ -1557,10 +1557,10 @@
         <v>52</v>
       </c>
       <c r="C42" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="D42" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
@@ -1571,10 +1571,10 @@
         <v>52</v>
       </c>
       <c r="C43" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="D43" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>